<commit_message>
DSP A类tag标注: Test/Sync/SyncCK/SyncManual/SyncV2/MSAccount 共73接口(按限制清单不生成不执行)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/single-api/dspapi/swagger_modules.xlsx
+++ b/single-api/dspapi/swagger_modules.xlsx
@@ -1686,9 +1686,19 @@
       </c>
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
+      <c r="F48" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>0% (0/3)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -33218,8 +33228,16 @@
         </is>
       </c>
       <c r="E1083" s="3" t="n"/>
-      <c r="F1083" s="3" t="n"/>
-      <c r="G1083" s="3" t="n"/>
+      <c r="F1083" s="5" t="inlineStr">
+        <is>
+          <t>不执行(A类限制)</t>
+        </is>
+      </c>
+      <c r="G1083" s="5" t="inlineStr">
+        <is>
+          <t>DSP限制清单A类：会影响account，不生成不执行</t>
+        </is>
+      </c>
     </row>
     <row r="1084">
       <c r="A1084" s="2" t="inlineStr">
@@ -33243,8 +33261,16 @@
         </is>
       </c>
       <c r="E1084" s="3" t="n"/>
-      <c r="F1084" s="3" t="n"/>
-      <c r="G1084" s="3" t="n"/>
+      <c r="F1084" s="5" t="inlineStr">
+        <is>
+          <t>不执行(A类限制)</t>
+        </is>
+      </c>
+      <c r="G1084" s="5" t="inlineStr">
+        <is>
+          <t>DSP限制清单A类：会影响account，不生成不执行</t>
+        </is>
+      </c>
     </row>
     <row r="1085">
       <c r="A1085" s="2" t="inlineStr">
@@ -33268,8 +33294,16 @@
         </is>
       </c>
       <c r="E1085" s="3" t="n"/>
-      <c r="F1085" s="3" t="n"/>
-      <c r="G1085" s="3" t="n"/>
+      <c r="F1085" s="5" t="inlineStr">
+        <is>
+          <t>不执行(A类限制)</t>
+        </is>
+      </c>
+      <c r="G1085" s="5" t="inlineStr">
+        <is>
+          <t>DSP限制清单A类：会影响account，不生成不执行</t>
+        </is>
+      </c>
     </row>
     <row r="1086">
       <c r="A1086" s="2" t="inlineStr">
@@ -43757,12 +43791,12 @@
       <c r="E1456" s="3" t="n"/>
       <c r="F1456" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1456" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43790,12 +43824,12 @@
       <c r="E1457" s="3" t="n"/>
       <c r="F1457" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1457" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43823,12 +43857,12 @@
       <c r="E1458" s="3" t="n"/>
       <c r="F1458" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1458" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43856,12 +43890,12 @@
       <c r="E1459" s="3" t="n"/>
       <c r="F1459" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1459" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43889,12 +43923,12 @@
       <c r="E1460" s="3" t="n"/>
       <c r="F1460" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1460" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43922,12 +43956,12 @@
       <c r="E1461" s="3" t="n"/>
       <c r="F1461" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1461" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43955,12 +43989,12 @@
       <c r="E1462" s="3" t="n"/>
       <c r="F1462" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1462" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -43988,12 +44022,12 @@
       <c r="E1463" s="3" t="n"/>
       <c r="F1463" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1463" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44021,12 +44055,12 @@
       <c r="E1464" s="3" t="n"/>
       <c r="F1464" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1464" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44054,12 +44088,12 @@
       <c r="E1465" s="3" t="n"/>
       <c r="F1465" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1465" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44087,12 +44121,12 @@
       <c r="E1466" s="3" t="n"/>
       <c r="F1466" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1466" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44120,12 +44154,12 @@
       <c r="E1467" s="3" t="n"/>
       <c r="F1467" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1467" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44153,12 +44187,12 @@
       <c r="E1468" s="3" t="n"/>
       <c r="F1468" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1468" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44186,12 +44220,12 @@
       <c r="E1469" s="3" t="n"/>
       <c r="F1469" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1469" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44219,12 +44253,12 @@
       <c r="E1470" s="3" t="n"/>
       <c r="F1470" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1470" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44252,12 +44286,12 @@
       <c r="E1471" s="3" t="n"/>
       <c r="F1471" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1471" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44285,12 +44319,12 @@
       <c r="E1472" s="3" t="n"/>
       <c r="F1472" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1472" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44318,12 +44352,12 @@
       <c r="E1473" s="3" t="n"/>
       <c r="F1473" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1473" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44351,12 +44385,12 @@
       <c r="E1474" s="3" t="n"/>
       <c r="F1474" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1474" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44384,12 +44418,12 @@
       <c r="E1475" s="3" t="n"/>
       <c r="F1475" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1475" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44417,12 +44451,12 @@
       <c r="E1476" s="3" t="n"/>
       <c r="F1476" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1476" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44450,12 +44484,12 @@
       <c r="E1477" s="3" t="n"/>
       <c r="F1477" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1477" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44483,12 +44517,12 @@
       <c r="E1478" s="3" t="n"/>
       <c r="F1478" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1478" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44516,12 +44550,12 @@
       <c r="E1479" s="3" t="n"/>
       <c r="F1479" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1479" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44549,12 +44583,12 @@
       <c r="E1480" s="3" t="n"/>
       <c r="F1480" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1480" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44582,12 +44616,12 @@
       <c r="E1481" s="3" t="n"/>
       <c r="F1481" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1481" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44615,12 +44649,12 @@
       <c r="E1482" s="3" t="n"/>
       <c r="F1482" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1482" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44648,12 +44682,12 @@
       <c r="E1483" s="3" t="n"/>
       <c r="F1483" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1483" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44681,12 +44715,12 @@
       <c r="E1484" s="3" t="n"/>
       <c r="F1484" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1484" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44714,12 +44748,12 @@
       <c r="E1485" s="3" t="n"/>
       <c r="F1485" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1485" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44747,12 +44781,12 @@
       <c r="E1486" s="3" t="n"/>
       <c r="F1486" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1486" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44780,12 +44814,12 @@
       <c r="E1487" s="3" t="n"/>
       <c r="F1487" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1487" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44813,12 +44847,12 @@
       <c r="E1488" s="3" t="n"/>
       <c r="F1488" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1488" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId；不排除clientId时有12次，全部来自clientId 0/62内部系统/自动化噪音)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44846,12 +44880,12 @@
       <c r="E1489" s="3" t="n"/>
       <c r="F1489" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1489" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId；不排除clientId时有7次，全部来自clientId 0/62内部系统/自动化噪音)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44879,12 +44913,12 @@
       <c r="E1490" s="3" t="n"/>
       <c r="F1490" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1490" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44912,12 +44946,12 @@
       <c r="E1491" s="3" t="n"/>
       <c r="F1491" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1491" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44945,12 +44979,12 @@
       <c r="E1492" s="3" t="n"/>
       <c r="F1492" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1492" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -44978,12 +45012,12 @@
       <c r="E1493" s="3" t="n"/>
       <c r="F1493" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1493" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词sync，不生成不执行(尽管365天399次真实流量，仍按硬性规则拦截)</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45011,12 +45045,12 @@
       <c r="E1494" s="3" t="n"/>
       <c r="F1494" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1494" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词sync，不生成不执行(尽管365天8328次真实流量，仍按硬性规则拦截)</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45044,12 +45078,12 @@
       <c r="E1495" s="3" t="n"/>
       <c r="F1495" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1495" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词sync，不生成不执行(尽管365天707次真实流量，仍按硬性规则拦截)</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45077,12 +45111,12 @@
       <c r="E1496" s="3" t="n"/>
       <c r="F1496" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1496" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45110,12 +45144,12 @@
       <c r="E1497" s="3" t="n"/>
       <c r="F1497" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1497" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45143,12 +45177,12 @@
       <c r="E1498" s="3" t="n"/>
       <c r="F1498" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1498" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -45176,12 +45210,12 @@
       <c r="E1499" s="3" t="n"/>
       <c r="F1499" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1499" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部从亚马逊拉数据，有上下文和执行顺序依赖，含只读GET也不跑</t>
         </is>
       </c>
     </row>
@@ -47110,12 +47144,12 @@
       <c r="E1566" s="3" t="n"/>
       <c r="F1566" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1566" s="5" t="inlineStr">
         <is>
-          <t>路径含禁用关键词test，不生成不执行(尽管365天8次真实流量，仍按硬性规则拦截)</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47143,12 +47177,12 @@
       <c r="E1567" s="3" t="n"/>
       <c r="F1567" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1567" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47176,12 +47210,12 @@
       <c r="E1568" s="3" t="n"/>
       <c r="F1568" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1568" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47209,12 +47243,12 @@
       <c r="E1569" s="3" t="n"/>
       <c r="F1569" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1569" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47242,12 +47276,12 @@
       <c r="E1570" s="3" t="n"/>
       <c r="F1570" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1570" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId；不排除clientId时有9次，全部来自clientId 0/62内部系统/自动化噪音)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47275,12 +47309,12 @@
       <c r="E1571" s="3" t="n"/>
       <c r="F1571" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1571" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47308,12 +47342,12 @@
       <c r="E1572" s="3" t="n"/>
       <c r="F1572" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1572" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47341,12 +47375,12 @@
       <c r="E1573" s="3" t="n"/>
       <c r="F1573" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1573" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47374,12 +47408,12 @@
       <c r="E1574" s="3" t="n"/>
       <c r="F1574" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1574" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47407,12 +47441,12 @@
       <c r="E1575" s="3" t="n"/>
       <c r="F1575" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1575" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47440,12 +47474,12 @@
       <c r="E1576" s="3" t="n"/>
       <c r="F1576" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1576" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47473,12 +47507,12 @@
       <c r="E1577" s="3" t="n"/>
       <c r="F1577" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1577" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47506,12 +47540,12 @@
       <c r="E1578" s="3" t="n"/>
       <c r="F1578" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1578" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47539,12 +47573,12 @@
       <c r="E1579" s="3" t="n"/>
       <c r="F1579" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1579" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47572,12 +47606,12 @@
       <c r="E1580" s="3" t="n"/>
       <c r="F1580" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1580" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47605,12 +47639,12 @@
       <c r="E1581" s="3" t="n"/>
       <c r="F1581" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1581" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47638,12 +47672,12 @@
       <c r="E1582" s="3" t="n"/>
       <c r="F1582" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1582" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47671,12 +47705,12 @@
       <c r="E1583" s="3" t="n"/>
       <c r="F1583" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1583" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47704,12 +47738,12 @@
       <c r="E1584" s="3" t="n"/>
       <c r="F1584" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1584" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47737,12 +47771,12 @@
       <c r="E1585" s="3" t="n"/>
       <c r="F1585" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1585" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47770,12 +47804,12 @@
       <c r="E1586" s="3" t="n"/>
       <c r="F1586" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1586" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47803,12 +47837,12 @@
       <c r="E1587" s="3" t="n"/>
       <c r="F1587" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1587" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47836,12 +47870,12 @@
       <c r="E1588" s="3" t="n"/>
       <c r="F1588" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1588" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47869,12 +47903,12 @@
       <c r="E1589" s="3" t="n"/>
       <c r="F1589" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1589" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47902,12 +47936,12 @@
       <c r="E1590" s="3" t="n"/>
       <c r="F1590" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1590" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>
@@ -47935,12 +47969,12 @@
       <c r="E1591" s="3" t="n"/>
       <c r="F1591" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量</t>
+          <t>不执行(A类限制)</t>
         </is>
       </c>
       <c r="G1591" s="5" t="inlineStr">
         <is>
-          <t>ES 无流量(365天0次，已排除测试clientId；不排除clientId时有12769032次，全部来自clientId 0/62内部系统/自动化噪音)，暂不覆盖</t>
+          <t>DSP限制清单A类：内部手动操作/测试用，用户不会直接用到，不生成不执行</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AttachFile/Research/AmcOAuth2 完成: 3个tag共3接口(AttachFile文件下载1个已执行/Research 2场景已执行两轮全PASS/AmcOAuth2因需真实一次性OAuth code技术受限未执行)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/single-api/dspapi/swagger_modules.xlsx
+++ b/single-api/dspapi/swagger_modules.xlsx
@@ -804,9 +804,19 @@
       </c>
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>0% (0/1)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -944,9 +954,19 @@
       </c>
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
-      <c r="H17" s="2" t="n"/>
+      <c r="F17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>100% (1/1)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2072,9 +2092,19 @@
       </c>
       <c r="D61" s="3" t="n"/>
       <c r="E61" s="3" t="n"/>
-      <c r="F61" s="2" t="n"/>
-      <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
+      <c r="F61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>100% (1/1)</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8171,8 +8201,16 @@
         </is>
       </c>
       <c r="E191" s="3" t="n"/>
-      <c r="F191" s="3" t="n"/>
-      <c r="G191" s="3" t="n"/>
+      <c r="F191" s="5" t="inlineStr">
+        <is>
+          <t>技术受限(需真实一次性OAuth code)</t>
+        </is>
+      </c>
+      <c r="G191" s="5" t="inlineStr">
+        <is>
+          <t>技术受限：该接口用于交换真实Amazon OAuth2一次性授权code换取AMC账号绑定，code是通过真实浏览器重定向流程获得的一次性凭证，无法在自动化测试中合法获取或重放；ES真实样本里的code均已被消费过，重放会因code已失效而报错，且该操作涉及真实向Amazon发起账号OAuth绑定请求，高风险不适合自动化测试。不生成不执行。</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -15086,7 +15124,7 @@
       <c r="F417" s="3" t="n"/>
       <c r="G417" s="3" t="n"/>
     </row>
-    <row r="418">
+    <row r="418" ht="16" customHeight="1">
       <c r="A418" s="2" t="inlineStr">
         <is>
           <t>us</t>
@@ -15108,7 +15146,11 @@
         </is>
       </c>
       <c r="E418" s="3" t="n"/>
-      <c r="F418" s="3" t="n"/>
+      <c r="F418" s="6" t="inlineStr">
+        <is>
+          <t>按RowGuid下载附件 — 100%</t>
+        </is>
+      </c>
       <c r="G418" s="3" t="n"/>
     </row>
     <row r="419">
@@ -41098,7 +41140,7 @@
         </is>
       </c>
     </row>
-    <row r="1336">
+    <row r="1336" ht="32" customHeight="1">
       <c r="A1336" s="2" t="inlineStr">
         <is>
           <t>us</t>
@@ -41120,7 +41162,12 @@
         </is>
       </c>
       <c r="E1336" s="3" t="n"/>
-      <c r="F1336" s="3" t="n"/>
+      <c r="F1336" s="6" t="inlineStr">
+        <is>
+          <t>不加类型/order过滤 — 74.0%
+同时加creativeTypes+orderIds过滤 — 7.2%</t>
+        </is>
+      </c>
       <c r="G1336" s="3" t="n"/>
     </row>
     <row r="1337">

</xml_diff>